<commit_message>
Merge wave 3: Eliza into Motto; Claim Check and Brain Blast into Expert Lens
</commit_message>
<xml_diff>
--- a/Nightly Runs/Project Portfolio.xlsx
+++ b/Nightly Runs/Project Portfolio.xlsx
@@ -3137,11 +3137,7 @@
           <t>finance-signals-dashboard</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>A standalone, Spark-hosted morning-briefing pipeline and private dashboard: at a configured cutoff it publishes one immutable "issue" with exact completed-session moves for six named equity indices (NIFTY 50, S&amp;P 500, Nikkei 225, KOSPI, STI, CSI 300) plus BTC/USD spot, deduplicated regional headlines, a deterministic template summary, and full evidence provenance. Serves one user via tailnet through Dashboard Command Center.</t>
-        </is>
-      </c>
+      <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr">
         <is>
           <t>Finance</t>
@@ -3154,7 +3150,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>FastAPI, Jinja, SQLite</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -3781,11 +3777,7 @@
           <t>expert-lens-skill</t>
         </is>
       </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>A local single-player knowledge game: start from a topic, hop six steps through surprising but source-backed Wikipedia/Wikidata connections (three choices per step), against a timer, ending in a shareable path card with facts and citations. The model never invents links — it only explains edges retrieved and validated from sources.</t>
-        </is>
-      </c>
+      <c r="D41" s="2" t="inlineStr"/>
       <c r="E41" s="2" t="inlineStr">
         <is>
           <t>Games</t>
@@ -3798,7 +3790,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Next.js, SQLite</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -4493,12 +4485,12 @@
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>absorbs batman-prep-time-skill, goal-to-calendar-planner, rabbit-hole-speedrun</t>
+          <t>absorbs batman-prep-time-skill, goal-to-calendar-planner, rabbit-hole-speedrun, physics-claim-debunker-skill, brain-blast-skill</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>**Expert Lens** (repo `expert-lens-skill`) is one private FirstSpark dashboard service. It turns "domain + situation + counterpart + outcome" into an evidence-backed **field card** (topology, vocabulary ladder with paraphrase tests, mechanism map, ranked expert questions, distinctions, rehearsal), and keeps every topic as a Markdown workspace you can read, edit and chat with through the owner's GLM 5.3 model. Merged features: **Batman Prep** (prep for any commitment, with Goal-to-Calendar planning as its approval-gated scheduling step) and **Rabbit Hole Speedrun** (a source-backed knowledge game that can start from a library topic). The Markdown library on disk is the source of truth and SQLite is a rebuildable index. It is deployed like YouTube Learning Center (YLC): a systemd user unit on `127.0.0.1:8767`, published at `https://spark-07a8.tail4a1242.ts.net:8767/` with Tailscale Serve, and shown as a tab in Dashboard Command Center (DCC).</t>
+          <t>**Expert Lens** (repo `expert-lens-skill`) is one private FirstSpark dashboard service. It turns "domain + situation + counterpart + outcome" into an evidence-backed **field card** (topology, vocabulary ladder with paraphrase tests, mechanism map, ranked expert questions, distinctions, rehearsal), and keeps every topic as a Markdown workspace you can read, edit and chat with through the owner's GLM 5.3 model. Merged features: **Batman Prep** (prep for any commitment, with Goal-to-Calendar planning as its approval-gated scheduling step) and **Rabbit Hole Speedrun** (a source-backed knowledge game that can start from a library topic). Also merged: **Claim Check** as the **Research** tab (a pasted claim becomes steelmanned physical subclaims tested with deterministic unit-aware code, a primary-source ledger that deliberately looks for contradicting measurements, and a six-way verdict) and **Brain Blast** as the **Experiments** tab (one everyday irritation becomes one cheap, reversible experiment, tracked as a shared `experiment.v1` card that this repo owns). The Markdown library on disk is the source of truth and SQLite is a rebuildable index. It is deployed like YouTube Learning Center (YLC): a systemd user unit on `127.0.0.1:8767`, published at `https://spark-07a8.tail4a1242.ts.net:8767/` with Tailscale Serve, and shown as a tab in Dashboard Command Center (DCC).</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -4559,7 +4551,7 @@
       <c r="P50" s="4" t="inlineStr"/>
       <c r="Q50" s="5" t="inlineStr">
         <is>
-          <t>1 blocking · 9 questions · 1 proposals</t>
+          <t>1 blocking · 15 questions · 2 proposals</t>
         </is>
       </c>
     </row>
@@ -5129,81 +5121,81 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="7" t="inlineStr">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>physics-claim-debunker-skill</t>
         </is>
       </c>
-      <c r="B58" s="7" t="inlineStr">
-        <is>
-          <t>Greenfield</t>
-        </is>
-      </c>
-      <c r="C58" s="7" t="inlineStr"/>
-      <c r="D58" s="7" t="inlineStr">
-        <is>
-          <t>A local research skill that turns an extraordinary claim into measurable subclaims, steelmans it, tests it with conservation laws, dimensions, orders of magnitude, geometry, and statistics via deterministic unit-aware code, compares predictions with primary measurements, and renders a layered (beginner/intermediate/technical) report with one of six verdict categories — including "unresolved" and "unfalsifiable as phrased". Value is the visible reasoning path, not a dramatic debunk.</t>
-        </is>
-      </c>
-      <c r="E58" s="7" t="inlineStr">
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Merged → feature</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>expert-lens-skill</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr"/>
+      <c r="E58" s="2" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="F58" s="7" t="inlineStr">
-        <is>
-          <t>Skill + CLI</t>
-        </is>
-      </c>
-      <c r="G58" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H58" s="7" t="inlineStr">
-        <is>
-          <t>Claude Code / Codex / Hermes</t>
-        </is>
-      </c>
-      <c r="I58" s="7" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="J58" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K58" s="7" t="inlineStr">
-        <is>
-          <t>Open-source</t>
-        </is>
-      </c>
-      <c r="L58" s="7" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="M58" s="7" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="N58" s="7" t="inlineStr">
-        <is>
-          <t>Deterministic, unit-aware claim checks: good open-source education.</t>
-        </is>
-      </c>
-      <c r="O58" s="8" t="inlineStr">
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>Feature of host</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M58" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N58" s="2" t="inlineStr">
+        <is>
+          <t>Research tab (Claim Check) of Expert Lens.</t>
+        </is>
+      </c>
+      <c r="O58" s="3" t="inlineStr">
         <is>
           <t>https://github.com/snknitin/physics-claim-debunker-skill</t>
         </is>
       </c>
       <c r="P58" s="4" t="inlineStr"/>
-      <c r="Q58" s="7" t="inlineStr">
-        <is>
-          <t>0 blocking · 1 questions · 0 proposals</t>
+      <c r="Q58" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -5460,11 +5452,7 @@
           <t>language-learning-lab</t>
         </is>
       </c>
-      <c r="D62" s="2" t="inlineStr">
-        <is>
-          <t>A personal Windows-first workbench that turns a vocabulary Google Sheet into durable context-to-word recall (reverse recall, FSRS-scheduled) and turns selected Handy dictations into evidence-linked speech coaching with a ten-minute daily drill. Single Windows writer; private models only; Markdown exports are selected artifacts, not the learning database.</t>
-        </is>
-      </c>
+      <c r="D62" s="2" t="inlineStr"/>
       <c r="E62" s="2" t="inlineStr">
         <is>
           <t>Learning</t>
@@ -5477,7 +5465,7 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>FastAPI, SQLite, React</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -5946,11 +5934,7 @@
           <t>expert-lens-skill</t>
         </is>
       </c>
-      <c r="D68" s="2" t="inlineStr">
-        <is>
-          <t>A Codex/Hermes skill that turns any pasted commitment (meeting, trip, exam, purchase, deadline, difficult conversation…) into the smallest high-signal preparation pack: mission, situation map, Pareto brief, backward plan, questions, pre-mortem, contingencies, and a ten-minute card — all inside a user-selected time budget. It can also take a Jobs Search and Apply Tool `interview-prep.json` as context for an interview.</t>
-        </is>
-      </c>
+      <c r="D68" s="2" t="inlineStr"/>
       <c r="E68" s="2" t="inlineStr">
         <is>
           <t>Personal ops</t>
@@ -6014,81 +5998,81 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="7" t="inlineStr">
+      <c r="A69" s="2" t="inlineStr">
         <is>
           <t>brain-blast-skill</t>
         </is>
       </c>
-      <c r="B69" s="7" t="inlineStr">
-        <is>
-          <t>Greenfield</t>
-        </is>
-      </c>
-      <c r="C69" s="7" t="inlineStr"/>
-      <c r="D69" s="7" t="inlineStr">
-        <is>
-          <t>A Markdown skill package that turns one everyday irritation into one cheap, reversible experiment: reframe the problem, apply a deterministic deck of creativity operators, score options, and emit a single experiment card plus an outcome log entry. Serves the owner's local agent (Claude Code / Codex / Hermes-style skill invocation).</t>
-        </is>
-      </c>
-      <c r="E69" s="7" t="inlineStr">
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Merged → feature</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>expert-lens-skill</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr"/>
+      <c r="E69" s="2" t="inlineStr">
         <is>
           <t>Personal ops</t>
         </is>
       </c>
-      <c r="F69" s="7" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="G69" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H69" s="7" t="inlineStr">
-        <is>
-          <t>Claude Code / Codex / Hermes</t>
-        </is>
-      </c>
-      <c r="I69" s="7" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="J69" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K69" s="7" t="inlineStr">
-        <is>
-          <t>Open-source</t>
-        </is>
-      </c>
-      <c r="L69" s="7" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="M69" s="7" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="N69" s="7" t="inlineStr">
-        <is>
-          <t>Small creativity skill.</t>
-        </is>
-      </c>
-      <c r="O69" s="8" t="inlineStr">
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>Feature of host</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="K69" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M69" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N69" s="2" t="inlineStr">
+        <is>
+          <t>Experiments tab (Brain Blast) of Expert Lens; owns experiment.v1.</t>
+        </is>
+      </c>
+      <c r="O69" s="3" t="inlineStr">
         <is>
           <t>https://github.com/snknitin/brain-blast-skill</t>
         </is>
       </c>
       <c r="P69" s="4" t="inlineStr"/>
-      <c r="Q69" s="7" t="inlineStr">
-        <is>
-          <t>0 blocking · 3 questions · 0 proposals</t>
+      <c r="Q69" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -6424,11 +6408,7 @@
           <t>expert-lens-skill</t>
         </is>
       </c>
-      <c r="D74" s="2" t="inlineStr">
-        <is>
-          <t>An approval-based local planner that turns one large goal into milestones and dependency-aware tasks, fits them into real free time with deliberate slack using a constraint solver, previews every week as a diff before any block exists, and replans from what actually happened — explaining every change. It is also the **owner of task/plan truth** that NPC Mode Coach and Jarvis and Alfred read (see §4 "Shared task truth").</t>
-        </is>
-      </c>
+      <c r="D74" s="2" t="inlineStr"/>
       <c r="E74" s="2" t="inlineStr">
         <is>
           <t>Personal ops</t>
@@ -6441,7 +6421,7 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Next.js, FastAPI, n8n, OR-Tools, Playwright, SQLite</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
@@ -6586,11 +6566,7 @@
           <t>motto-agent-council</t>
         </is>
       </c>
-      <c r="D76" s="2" t="inlineStr">
-        <is>
-          <t>A two-role personal executive-assistant harness: Jarvis turns requests into bounded, previewed tasks and drafts; Alfred maintains the morning brief/weekly review and challenges overload. Both share one structured memory with provenance and one authority model — personality never changes authority. Calendar and task data are read from the same sources Goal-to-Calendar Planner and NPC Mode Coach use; this harness never owns task truth.</t>
-        </is>
-      </c>
+      <c r="D76" s="2" t="inlineStr"/>
       <c r="E76" s="2" t="inlineStr">
         <is>
           <t>Personal ops</t>
@@ -6603,7 +6579,7 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>FastAPI, HTMX, LangGraph, SQLite</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
@@ -6745,12 +6721,12 @@
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>absorbs jarvis-and-alfred, parallel-presence-companions</t>
+          <t>absorbs jarvis-and-alfred, parallel-presence-companions, reflective-eliza-companion</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>A local council of small, explicit perspective agents — each a user-authored charter (builder, skeptic, health protector…) — that critique one decision from identical facts, label every claim as fact/assumption/value/unknown, challenge each other for one bounded round, and yield a chair memo that preserves dissent. It corrects charters from outcomes; it never pretends to be a digital twin. Later (README "voice/persona presentation"), the council can present itself as owner-designed characters, each with its own Voice Studio voice, holding a spoken discussion of the owner's decision with him, grounded in his motto and philosophy. Merged features (owner direction 2026-10-20): the characters live as small always-on-top **desktop pets** on the Windows desktop; **Jarvis and Alfred** (from `features/jarvis-and-alfred/`) are two resident council voices with executive-assistant duties over calendar and tasks (read-only, drafts behind approval); **Parallel Presence Companions** (from `features/parallel-presence-companions/`) become pet-hosted body-doubling focus sessions; the council core stays a headless, testable Python CLI + local API.</t>
+          <t>A local council of small, explicit perspective agents — each a user-authored charter (builder, skeptic, health protector…) — that critique one decision from identical facts, label every claim as fact/assumption/value/unknown, challenge each other for one bounded round, and yield a chair memo that preserves dissent. It corrects charters from outcomes; it never pretends to be a digital twin. Later (README "voice/persona presentation"), the council can present itself as owner-designed characters, each with its own Voice Studio voice, holding a spoken discussion of the owner's decision with him, grounded in his motto and philosophy. Merged features (owner direction 2026-10-20): the characters live as small always-on-top **desktop pets** on the Windows desktop; **Jarvis and Alfred** (from `features/jarvis-and-alfred/`) are two resident council voices with executive-assistant duties over calendar and tasks (read-only, drafts behind approval); **Parallel Presence Companions** (from `features/parallel-presence-companions/`) become pet-hosted body-doubling focus sessions; the council core stays a headless, testable Python CLI + local API. **Reflective Eliza** (from `features/reflective-eliza-companion/`, owner direction 2026-10-20) joins as a listening council character with six conversation modes in a desktop chat window; it writes owner-confirmed reflective memory and `experiment.v1` cards into the one shared memory store (host T18–T19) that Jarvis, Alfred and the focus companions also use.</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -6800,7 +6776,7 @@
       </c>
       <c r="N78" s="5" t="inlineStr">
         <is>
-          <t>Multi-voice council; Jarvis/Alfred desktop pets voiced by Voice Studio; body-doubling focus sessions.</t>
+          <t>Multi-voice council; Jarvis/Alfred desktop pets voiced by Voice Studio; body-doubling focus sessions; Eliza reflective companion. Ideas ported from angel-and-demon-companion.</t>
         </is>
       </c>
       <c r="O78" s="6" t="inlineStr">
@@ -6811,7 +6787,7 @@
       <c r="P78" s="4" t="inlineStr"/>
       <c r="Q78" s="5" t="inlineStr">
         <is>
-          <t>3 blocking · 8 questions · 4 proposals</t>
+          <t>4 blocking · 15 questions · 6 proposals</t>
         </is>
       </c>
     </row>
@@ -6831,11 +6807,7 @@
           <t>paper-logbook</t>
         </is>
       </c>
-      <c r="D79" s="2" t="inlineStr">
-        <is>
-          <t>A playful, local-first daily coach that compares today's actual behavior with a user-authored "ideal player character" (chosen values + repeatable behaviors), turns the biggest gap into one executable quest chain, and drafts low-risk admin actions for approval. Momentum, not shame: comparison language describes state ("two tasks are blocked"), never identity. Per README it is a **view over the same task truth as Goal-to-Calendar Planner**, not a second task system.</t>
-        </is>
-      </c>
+      <c r="D79" s="2" t="inlineStr"/>
       <c r="E79" s="2" t="inlineStr">
         <is>
           <t>Personal ops</t>
@@ -6848,7 +6820,7 @@
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>Expo, FastAPI, OR-Tools, SQLite</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
@@ -6997,11 +6969,7 @@
           <t>motto-agent-council</t>
         </is>
       </c>
-      <c r="D81" s="2" t="inlineStr">
-        <is>
-          <t>A body-doubling focus room: the user declares the next visible task, runs a session with either a real partner or a clearly-labeled synthetic original character, gets lightweight checkpoint check-ins (progress / blocker / next action), and ends with a receipt. Ambient presence, not conversation.</t>
-        </is>
-      </c>
+      <c r="D81" s="2" t="inlineStr"/>
       <c r="E81" s="2" t="inlineStr">
         <is>
           <t>Personal ops</t>
@@ -7014,7 +6982,7 @@
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>SvelteKit, Tauri, SQLite</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
@@ -7385,81 +7353,81 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="7" t="inlineStr">
+      <c r="A86" s="2" t="inlineStr">
         <is>
           <t>reflective-eliza-companion</t>
         </is>
       </c>
-      <c r="B86" s="7" t="inlineStr">
-        <is>
-          <t>Greenfield</t>
-        </is>
-      </c>
-      <c r="C86" s="7" t="inlineStr"/>
-      <c r="D86" s="7" t="inlineStr">
-        <is>
-          <t>A private, local-first reflective conversation companion: ELIZA-style listening backed by durable, user-auditable memory (facts, preferences, hypotheses, open threads, experiments), with every inference revisable and deletable. It serves one user on their own machine. It must never claim clinical authority, conceal model uncertainty, or optimize for longer or more frequent chats — sessions end in an optional action, not a hook.</t>
-        </is>
-      </c>
-      <c r="E86" s="7" t="inlineStr">
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>Merged → feature</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>motto-agent-council</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr"/>
+      <c r="E86" s="2" t="inlineStr">
         <is>
           <t>Personal ops</t>
         </is>
       </c>
-      <c r="F86" s="7" t="inlineStr">
-        <is>
-          <t>Desktop app (Tauri)</t>
-        </is>
-      </c>
-      <c r="G86" s="7" t="inlineStr">
-        <is>
-          <t>Tauri, SQLite</t>
-        </is>
-      </c>
-      <c r="H86" s="7" t="inlineStr">
-        <is>
-          <t>Windows desktop</t>
-        </is>
-      </c>
-      <c r="I86" s="7" t="inlineStr">
-        <is>
-          <t>Standalone desktop</t>
-        </is>
-      </c>
-      <c r="J86" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K86" s="7" t="inlineStr">
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
+          <t>Feature of host</t>
+        </is>
+      </c>
+      <c r="J86" s="2" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="L86" s="7" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="M86" s="7" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="N86" s="7" t="inlineStr">
-        <is>
-          <t>Private reflective companion; sensitive, keep personal.</t>
-        </is>
-      </c>
-      <c r="O86" s="8" t="inlineStr">
+      <c r="K86" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L86" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M86" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N86" s="2" t="inlineStr">
+        <is>
+          <t>Eliza listening character inside Motto; memory merged into the shared store.</t>
+        </is>
+      </c>
+      <c r="O86" s="3" t="inlineStr">
         <is>
           <t>https://github.com/snknitin/reflective-eliza-companion</t>
         </is>
       </c>
       <c r="P86" s="4" t="inlineStr"/>
-      <c r="Q86" s="7" t="inlineStr">
-        <is>
-          <t>1 blocking · 3 questions · 0 proposals</t>
+      <c r="Q86" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -8119,11 +8087,7 @@
           <t>creator-content-engine</t>
         </is>
       </c>
-      <c r="D95" s="2" t="inlineStr">
-        <is>
-          <t>A local-first writing desk that drafts public posts (X, LinkedIn) and private DM replies in the owner's actual voice, grounded in curated Obsidian/Notion sources with heading-level provenance, relationship cards with promises/open loops, and an inspectable voice card that learns from accepted edit diffs. Every factual/personal claim cites a source or is flagged for user input. Public and private modes share the voice primitives but never each other's data.</t>
-        </is>
-      </c>
+      <c r="D95" s="2" t="inlineStr"/>
       <c r="E95" s="2" t="inlineStr">
         <is>
           <t>Publishing</t>
@@ -8136,7 +8100,7 @@
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>SvelteKit, FastAPI, SQLite</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
@@ -9237,11 +9201,7 @@
           <t>creator-content-engine</t>
         </is>
       </c>
-      <c r="D109" s="2" t="inlineStr">
-        <is>
-          <t>A local review-and-apply workflow that audits everything you follow (YouTube + one other platform), builds a source registry with activity/topic/value evidence, and proposes a reversible keep/list/sample-less/archive/mute/review/unsubscribe plan — archiving cornerstone content from valuable sources *before* anything is removed. Changes are applied manually first from an exported checklist. This project owns the **source portfolio** (who/what you follow). Merged feature: **X Lists** (former X Like-to-List Builder) — X is the curator's second platform, and its X module clusters your X likes into 5–12 reviewed, export-only X List proposals.</t>
-        </is>
-      </c>
+      <c r="D109" s="2" t="inlineStr"/>
       <c r="E109" s="2" t="inlineStr">
         <is>
           <t>Signals</t>
@@ -9254,7 +9214,7 @@
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>Streamlit, sentence-transformers, Polars, SQLite</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H109" s="2" t="inlineStr">
@@ -9399,11 +9359,7 @@
           <t>creator-content-engine</t>
         </is>
       </c>
-      <c r="D111" s="2" t="inlineStr">
-        <is>
-          <t>A local pipeline + transcript-first editor that analyzes a long video (MP4/MKV/MOV), proposes standalone high-value segments via an explicit editable rubric, and renders approved ranges as 9:16 clips with accurate captions, clean boundaries, and complete provenance — never modifying the source. Deterministic editing of real footage; generative assets are explicitly not the core. Merged feature: **Podcast Clips** (former Podcast Clips Agency) — an audio/podcast input profile of the same pipeline that adds ownership attestation, context-checked moment scoring, audiogram 9:16 clips, copy drafts, and a publication manifest; export stays manual.</t>
-        </is>
-      </c>
+      <c r="D111" s="2" t="inlineStr"/>
       <c r="E111" s="2" t="inlineStr">
         <is>
           <t>Studio</t>
@@ -9416,7 +9372,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>SvelteKit, FastAPI, PyTorch, FFmpeg, SQLite</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -10513,11 +10469,7 @@
           <t>moving-out-marketplace</t>
         </is>
       </c>
-      <c r="D125" s="2" t="inlineStr">
-        <is>
-          <t>A local web app that turns room photos into a user-correctable item inventory with conservative resale ranges backed by traceable comparable links the user pastes. Output is evidence — detections, corrections, assumptions, comparables, low/median/high ranges with sample sizes — never one magical total.</t>
-        </is>
-      </c>
+      <c r="D125" s="2" t="inlineStr"/>
       <c r="E125" s="2" t="inlineStr">
         <is>
           <t>Utilities</t>
@@ -10530,7 +10482,7 @@
       </c>
       <c r="G125" s="2" t="inlineStr">
         <is>
-          <t>FastAPI, HTMX, Jinja, SQLite</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H125" s="2" t="inlineStr">
@@ -11862,7 +11814,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D48"/>
+  <dimension ref="A1:D51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -12270,51 +12222,51 @@
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>understand-this-paper</t>
+          <t>physics-claim-debunker-skill</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>Built elsewhere</t>
+          <t>Merged → feature</t>
         </is>
       </c>
       <c r="C19" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>expert-lens-skill</t>
         </is>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
-          <t>Almost complete hackathon build; remaining work is extension packaging + open-sourcing.</t>
+          <t>Research tab (Claim Check) of Expert Lens.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>vocabulary-diction-studio</t>
+          <t>understand-this-paper</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>Merged → feature</t>
+          <t>Built elsewhere</t>
         </is>
       </c>
       <c r="C20" s="14" t="inlineStr">
         <is>
-          <t>language-learning-lab</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D20" s="14" t="inlineStr">
         <is>
-          <t>English track of the Language Learning Lab.</t>
+          <t>Almost complete hackathon build; remaining work is extension packaging + open-sourcing.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>quiz-poker</t>
+          <t>vocabulary-diction-studio</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
@@ -12324,63 +12276,63 @@
       </c>
       <c r="C21" s="14" t="inlineStr">
         <is>
-          <t>quiz-master</t>
+          <t>language-learning-lab</t>
         </is>
       </c>
       <c r="D21" s="14" t="inlineStr">
         <is>
-          <t>Game tab inside Quiz Master.</t>
+          <t>English track of the Language Learning Lab.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>angel-and-demon-companion</t>
+          <t>quiz-poker</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
         <is>
-          <t>Kept (ideas ported)</t>
+          <t>Merged → feature</t>
         </is>
       </c>
       <c r="C22" s="14" t="inlineStr">
         <is>
-          <t>motto-agent-council</t>
+          <t>quiz-master</t>
         </is>
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
-          <t>Half-day hackathon site; ideas now live in Motto Council; repo left alone.</t>
+          <t>Game tab inside Quiz Master.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>batman-prep-time-skill</t>
+          <t>angel-and-demon-companion</t>
         </is>
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>Merged → feature</t>
+          <t>Kept (ideas ported)</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr">
         <is>
-          <t>expert-lens-skill</t>
+          <t>motto-agent-council</t>
         </is>
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>
-          <t>Batman Prep tab of Expert Lens.</t>
+          <t>Half-day hackathon site; ideas now live in Motto Council; repo left alone.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>brainrot-rehab</t>
+          <t>batman-prep-time-skill</t>
         </is>
       </c>
       <c r="B24" s="14" t="inlineStr">
@@ -12390,19 +12342,19 @@
       </c>
       <c r="C24" s="14" t="inlineStr">
         <is>
-          <t>paper-logbook</t>
+          <t>expert-lens-skill</t>
         </is>
       </c>
       <c r="D24" s="14" t="inlineStr">
         <is>
-          <t>Screen-time experiment pack inside Paper Logbook.</t>
+          <t>Batman Prep tab of Expert Lens.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>goal-to-calendar-planner</t>
+          <t>brain-blast-skill</t>
         </is>
       </c>
       <c r="B25" s="14" t="inlineStr">
@@ -12417,14 +12369,14 @@
       </c>
       <c r="D25" s="14" t="inlineStr">
         <is>
-          <t>Plan step inside the Batman Prep tab; g2c.tasks.v1 now served by Expert Lens.</t>
+          <t>Experiments tab (Brain Blast) of Expert Lens; owns experiment.v1.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>jarvis-and-alfred</t>
+          <t>brainrot-rehab</t>
         </is>
       </c>
       <c r="B26" s="14" t="inlineStr">
@@ -12434,19 +12386,19 @@
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>motto-agent-council</t>
+          <t>paper-logbook</t>
         </is>
       </c>
       <c r="D26" s="14" t="inlineStr">
         <is>
-          <t>Jarvis and Alfred become council voices / desktop pets.</t>
+          <t>Screen-time experiment pack inside Paper Logbook.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="14" t="inlineStr">
         <is>
-          <t>measure-life</t>
+          <t>goal-to-calendar-planner</t>
         </is>
       </c>
       <c r="B27" s="14" t="inlineStr">
@@ -12456,19 +12408,19 @@
       </c>
       <c r="C27" s="14" t="inlineStr">
         <is>
-          <t>paper-logbook</t>
+          <t>expert-lens-skill</t>
         </is>
       </c>
       <c r="D27" s="14" t="inlineStr">
         <is>
-          <t>Insights &amp; experiments tab inside Paper Logbook.</t>
+          <t>Plan step inside the Batman Prep tab; g2c.tasks.v1 now served by Expert Lens.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>npc-mode-personal-coach</t>
+          <t>jarvis-and-alfred</t>
         </is>
       </c>
       <c r="B28" s="14" t="inlineStr">
@@ -12478,19 +12430,19 @@
       </c>
       <c r="C28" s="14" t="inlineStr">
         <is>
-          <t>paper-logbook</t>
+          <t>motto-agent-council</t>
         </is>
       </c>
       <c r="D28" s="14" t="inlineStr">
         <is>
-          <t>NPC Mode interstitial-journaling tab of Paper Logbook.</t>
+          <t>Jarvis and Alfred become council voices / desktop pets.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="14" t="inlineStr">
         <is>
-          <t>parallel-presence-companions</t>
+          <t>measure-life</t>
         </is>
       </c>
       <c r="B29" s="14" t="inlineStr">
@@ -12500,41 +12452,41 @@
       </c>
       <c r="C29" s="14" t="inlineStr">
         <is>
-          <t>motto-agent-council</t>
+          <t>paper-logbook</t>
         </is>
       </c>
       <c r="D29" s="14" t="inlineStr">
         <is>
-          <t>Body doubling via the always-on desktop pets.</t>
+          <t>Insights &amp; experiments tab inside Paper Logbook.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>pocket-crm</t>
+          <t>npc-mode-personal-coach</t>
         </is>
       </c>
       <c r="B30" s="14" t="inlineStr">
         <is>
-          <t>Parked (archived)</t>
+          <t>Merged → feature</t>
         </is>
       </c>
       <c r="C30" s="14" t="inlineStr">
         <is>
-          <t>dunbar-dossier (idea note)</t>
+          <t>paper-logbook</t>
         </is>
       </c>
       <c r="D30" s="14" t="inlineStr">
         <is>
-          <t>Future Telegram capture front-end for dunbar-dossier.</t>
+          <t>NPC Mode interstitial-journaling tab of Paper Logbook.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>build-in-public-autoposter</t>
+          <t>parallel-presence-companions</t>
         </is>
       </c>
       <c r="B31" s="14" t="inlineStr">
@@ -12544,41 +12496,41 @@
       </c>
       <c r="C31" s="14" t="inlineStr">
         <is>
-          <t>creator-content-engine</t>
+          <t>motto-agent-council</t>
         </is>
       </c>
       <c r="D31" s="14" t="inlineStr">
         <is>
-          <t>Git-activity idea source.</t>
+          <t>Body doubling via the always-on desktop pets.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="14" t="inlineStr">
         <is>
-          <t>my-agent-posts-about-me</t>
+          <t>pocket-crm</t>
         </is>
       </c>
       <c r="B32" s="14" t="inlineStr">
         <is>
-          <t>Merged → feature</t>
+          <t>Parked (archived)</t>
         </is>
       </c>
       <c r="C32" s="14" t="inlineStr">
         <is>
-          <t>creator-content-engine</t>
+          <t>dunbar-dossier (idea note)</t>
         </is>
       </c>
       <c r="D32" s="14" t="inlineStr">
         <is>
-          <t>Daily-log idea source.</t>
+          <t>Future Telegram capture front-end for dunbar-dossier.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="14" t="inlineStr">
         <is>
-          <t>personal-voice-ghostwriter-and-dm-desk</t>
+          <t>reflective-eliza-companion</t>
         </is>
       </c>
       <c r="B33" s="14" t="inlineStr">
@@ -12588,19 +12540,19 @@
       </c>
       <c r="C33" s="14" t="inlineStr">
         <is>
-          <t>creator-content-engine</t>
+          <t>motto-agent-council</t>
         </is>
       </c>
       <c r="D33" s="14" t="inlineStr">
         <is>
-          <t>Voice + DM desk of Creator Content Engine.</t>
+          <t>Eliza listening character inside Motto; memory merged into the shared store.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
         <is>
-          <t>roast-my-landing-page</t>
+          <t>build-in-public-autoposter</t>
         </is>
       </c>
       <c r="B34" s="14" t="inlineStr">
@@ -12610,19 +12562,19 @@
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>landing-page-conversion-agency</t>
+          <t>creator-content-engine</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>Roast mode share card.</t>
+          <t>Git-activity idea source.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="14" t="inlineStr">
         <is>
-          <t>x-profile-autopsy</t>
+          <t>my-agent-posts-about-me</t>
         </is>
       </c>
       <c r="B35" s="14" t="inlineStr">
@@ -12637,58 +12589,58 @@
       </c>
       <c r="D35" s="14" t="inlineStr">
         <is>
-          <t>Profile-analysis tab.</t>
+          <t>Daily-log idea source.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="14" t="inlineStr">
         <is>
-          <t>personal-signal-intelligence-os</t>
+          <t>personal-voice-ghostwriter-and-dm-desk</t>
         </is>
       </c>
       <c r="B36" s="14" t="inlineStr">
         <is>
-          <t>Parked (archived)</t>
+          <t>Merged → feature</t>
         </is>
       </c>
       <c r="C36" s="14" t="inlineStr">
         <is>
-          <t>fresh-brief (idea note)</t>
+          <t>creator-content-engine</t>
         </is>
       </c>
       <c r="D36" s="14" t="inlineStr">
         <is>
-          <t>Duplicate of fresh-brief.</t>
+          <t>Voice + DM desk of Creator Content Engine.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="14" t="inlineStr">
         <is>
-          <t>shortform-signal-digest</t>
+          <t>roast-my-landing-page</t>
         </is>
       </c>
       <c r="B37" s="14" t="inlineStr">
         <is>
-          <t>Parked (archived)</t>
+          <t>Merged → feature</t>
         </is>
       </c>
       <c r="C37" s="14" t="inlineStr">
         <is>
-          <t>fresh-brief (idea note)</t>
+          <t>landing-page-conversion-agency</t>
         </is>
       </c>
       <c r="D37" s="14" t="inlineStr">
         <is>
-          <t>Future short-form desk for fresh-brief.</t>
+          <t>Roast mode share card.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t>social-subscription-curator</t>
+          <t>x-profile-autopsy</t>
         </is>
       </c>
       <c r="B38" s="14" t="inlineStr">
@@ -12703,58 +12655,58 @@
       </c>
       <c r="D38" s="14" t="inlineStr">
         <is>
-          <t>Follow portfolio area of Creator Content Engine.</t>
+          <t>Profile-analysis tab.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="14" t="inlineStr">
         <is>
-          <t>x-like-to-list-builder</t>
+          <t>personal-signal-intelligence-os</t>
         </is>
       </c>
       <c r="B39" s="14" t="inlineStr">
         <is>
-          <t>Merged → feature</t>
+          <t>Parked (archived)</t>
         </is>
       </c>
       <c r="C39" s="14" t="inlineStr">
         <is>
-          <t>social-subscription-curator</t>
+          <t>fresh-brief (idea note)</t>
         </is>
       </c>
       <c r="D39" s="14" t="inlineStr">
         <is>
-          <t>X module of the curator.</t>
+          <t>Duplicate of fresh-brief.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="14" t="inlineStr">
         <is>
-          <t>longform-to-shorts-studio</t>
+          <t>shortform-signal-digest</t>
         </is>
       </c>
       <c r="B40" s="14" t="inlineStr">
         <is>
-          <t>Merged → feature</t>
+          <t>Parked (archived)</t>
         </is>
       </c>
       <c r="C40" s="14" t="inlineStr">
         <is>
-          <t>creator-content-engine</t>
+          <t>fresh-brief (idea note)</t>
         </is>
       </c>
       <c r="D40" s="14" t="inlineStr">
         <is>
-          <t>Studio area of Creator Content Engine.</t>
+          <t>Future short-form desk for fresh-brief.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="14" t="inlineStr">
         <is>
-          <t>podcast-clips-agency</t>
+          <t>social-subscription-curator</t>
         </is>
       </c>
       <c r="B41" s="14" t="inlineStr">
@@ -12764,41 +12716,41 @@
       </c>
       <c r="C41" s="14" t="inlineStr">
         <is>
-          <t>longform-to-shorts-studio</t>
+          <t>creator-content-engine</t>
         </is>
       </c>
       <c r="D41" s="14" t="inlineStr">
         <is>
-          <t>Podcast input profile.</t>
+          <t>Follow portfolio area of Creator Content Engine.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="14" t="inlineStr">
         <is>
-          <t>agent-reach</t>
+          <t>x-like-to-list-builder</t>
         </is>
       </c>
       <c r="B42" s="14" t="inlineStr">
         <is>
-          <t>Third-party</t>
+          <t>Merged → feature</t>
         </is>
       </c>
       <c r="C42" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>social-subscription-curator</t>
         </is>
       </c>
       <c r="D42" s="14" t="inlineStr">
         <is>
-          <t>Open-source project you use; not yours, excluded from portfolio work.</t>
+          <t>X module of the curator.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="14" t="inlineStr">
         <is>
-          <t>price-my-room</t>
+          <t>longform-to-shorts-studio</t>
         </is>
       </c>
       <c r="B43" s="14" t="inlineStr">
@@ -12808,19 +12760,19 @@
       </c>
       <c r="C43" s="14" t="inlineStr">
         <is>
-          <t>moving-out-marketplace</t>
+          <t>creator-content-engine</t>
         </is>
       </c>
       <c r="D43" s="14" t="inlineStr">
         <is>
-          <t>Photo-to-price intake of the move-out storefront.</t>
+          <t>Studio area of Creator Content Engine.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="14" t="inlineStr">
         <is>
-          <t>b2b-competitor-battlecard</t>
+          <t>podcast-clips-agency</t>
         </is>
       </c>
       <c r="B44" s="14" t="inlineStr">
@@ -12830,41 +12782,41 @@
       </c>
       <c r="C44" s="14" t="inlineStr">
         <is>
-          <t>competitive-intelligence-agency</t>
+          <t>longform-to-shorts-studio</t>
         </is>
       </c>
       <c r="D44" s="14" t="inlineStr">
         <is>
-          <t>Battlecard export of the evidence library.</t>
+          <t>Podcast input profile.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="14" t="inlineStr">
         <is>
-          <t>cold-email-rewrite-desk</t>
+          <t>agent-reach</t>
         </is>
       </c>
       <c r="B45" s="14" t="inlineStr">
         <is>
-          <t>Merged → feature</t>
+          <t>Third-party</t>
         </is>
       </c>
       <c r="C45" s="14" t="inlineStr">
         <is>
-          <t>sales-development-agency</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D45" s="14" t="inlineStr">
         <is>
-          <t>Rewrite-desk tab.</t>
+          <t>Open-source project you use; not yours, excluded from portfolio work.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
-          <t>conversion-list-builder</t>
+          <t>price-my-room</t>
         </is>
       </c>
       <c r="B46" s="14" t="inlineStr">
@@ -12874,19 +12826,19 @@
       </c>
       <c r="C46" s="14" t="inlineStr">
         <is>
-          <t>demand-generation-workbench</t>
+          <t>moving-out-marketplace</t>
         </is>
       </c>
       <c r="D46" s="14" t="inlineStr">
         <is>
-          <t>Audience tab.</t>
+          <t>Photo-to-price intake of the move-out storefront.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="14" t="inlineStr">
         <is>
-          <t>linkedin-lead-list-plus-first-lines</t>
+          <t>b2b-competitor-battlecard</t>
         </is>
       </c>
       <c r="B47" s="14" t="inlineStr">
@@ -12896,32 +12848,98 @@
       </c>
       <c r="C47" s="14" t="inlineStr">
         <is>
-          <t>sales-development-agency</t>
+          <t>competitive-intelligence-agency</t>
         </is>
       </c>
       <c r="D47" s="14" t="inlineStr">
         <is>
-          <t>Prospect-CSV + first-lines feature.</t>
+          <t>Battlecard export of the evidence library.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="14" t="inlineStr">
         <is>
+          <t>cold-email-rewrite-desk</t>
+        </is>
+      </c>
+      <c r="B48" s="14" t="inlineStr">
+        <is>
+          <t>Merged → feature</t>
+        </is>
+      </c>
+      <c r="C48" s="14" t="inlineStr">
+        <is>
+          <t>sales-development-agency</t>
+        </is>
+      </c>
+      <c r="D48" s="14" t="inlineStr">
+        <is>
+          <t>Rewrite-desk tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="14" t="inlineStr">
+        <is>
+          <t>conversion-list-builder</t>
+        </is>
+      </c>
+      <c r="B49" s="14" t="inlineStr">
+        <is>
+          <t>Merged → feature</t>
+        </is>
+      </c>
+      <c r="C49" s="14" t="inlineStr">
+        <is>
+          <t>demand-generation-workbench</t>
+        </is>
+      </c>
+      <c r="D49" s="14" t="inlineStr">
+        <is>
+          <t>Audience tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="14" t="inlineStr">
+        <is>
+          <t>linkedin-lead-list-plus-first-lines</t>
+        </is>
+      </c>
+      <c r="B50" s="14" t="inlineStr">
+        <is>
+          <t>Merged → feature</t>
+        </is>
+      </c>
+      <c r="C50" s="14" t="inlineStr">
+        <is>
+          <t>sales-development-agency</t>
+        </is>
+      </c>
+      <c r="D50" s="14" t="inlineStr">
+        <is>
+          <t>Prospect-CSV + first-lines feature.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="14" t="inlineStr">
+        <is>
           <t>startup-graveyard</t>
         </is>
       </c>
-      <c r="B48" s="14" t="inlineStr">
+      <c r="B51" s="14" t="inlineStr">
         <is>
           <t>Merged → feature</t>
         </is>
       </c>
-      <c r="C48" s="14" t="inlineStr">
+      <c r="C51" s="14" t="inlineStr">
         <is>
           <t>side-hustle-radar</t>
         </is>
       </c>
-      <c r="D48" s="14" t="inlineStr">
+      <c r="D51" s="14" t="inlineStr">
         <is>
           <t>Failure-research tab.</t>
         </is>

</xml_diff>